<commit_message>
feat: Power query ETL tips
</commit_message>
<xml_diff>
--- a/Proyectos/Proyecto8 - Funciones Adicionales de Power BI/Recursos/1+-+Ejemplos/E1.xlsx
+++ b/Proyectos/Proyecto8 - Funciones Adicionales de Power BI/Recursos/1+-+Ejemplos/E1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\1 - Ejemplos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\Computacion\Data\Analytics\Udemy\Power BI\Curso Power BI – Análisis de Datos y Business Intelligence\Proyectos\Proyecto8 - Funciones Adicionales de Power BI\Recursos\1+-+Ejemplos\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647CB4C0-9C15-460E-81C2-E3B41D5D03A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="9576"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="9" r:id="rId1"/>
@@ -195,7 +196,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -521,7 +522,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -729,30 +730,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color theme="1" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color theme="1" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -778,127 +755,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.44999542222357858"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.44999542222357858"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color theme="0" tint="-0.34998626667073579"/>
       </top>
@@ -961,6 +821,81 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.44999542222357858"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.44999542222357858"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1006,83 +941,361 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.44999542222357858"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="1" tint="0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1" tint="0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1093,6 +1306,29 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B8048242-E604-4C79-81A5-6CE7BDC5CC6E}" name="Tabla1" displayName="Tabla1" ref="B3:O164" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="15" tableBorderDxfId="16">
+  <autoFilter ref="B3:O164" xr:uid="{B8048242-E604-4C79-81A5-6CE7BDC5CC6E}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{AC5C5D0F-CAE8-4FD5-824F-894A9C60453C}" name="Año" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{263B5DCD-2378-4EE1-8B13-E20479234E6B}" name="Genero" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{8D465A32-34E6-456D-93DA-5CEB86B3052D}" name="ene" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{5819C185-245E-4A38-A4D9-C4910CBA8A3B}" name="feb" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{CD859846-B5E5-4F7F-B3F1-B5F75924BD96}" name="mar" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{532140CA-633B-4570-A2B0-3B6C32434907}" name="abr" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{738A6195-FB87-482B-9667-F8D3C7AE523B}" name="may" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{0DD6B93F-117D-491A-B2CA-F8F7E9DF1601}" name="jun" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{7896AEAA-5187-42D6-9F87-F853C699F72B}" name="jul" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{AF8479E3-135F-4D22-B502-B329B86E98DD}" name="ago" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{4AE23149-1CE0-4011-A10C-EF15A68D8019}" name="sep" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{B2EA346E-0EC4-4F57-949C-B57CF4D2B578}" name="oct" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{33B998A0-7810-4531-95A3-B781D73632E9}" name="nov" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{C75CFE35-446F-40C3-A104-FF25DFABCC1F}" name="dic" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1357,97 +1593,98 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:T166"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" style="22"/>
-    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="3.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.88671875" style="22"/>
+    <col min="1" max="1" width="3.28515625" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5703125" customWidth="1"/>
+    <col min="5" max="5" width="6.140625" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="8" max="8" width="6.85546875" customWidth="1"/>
+    <col min="9" max="9" width="6" customWidth="1"/>
+    <col min="10" max="10" width="5.42578125" customWidth="1"/>
+    <col min="11" max="12" width="6.28515625" customWidth="1"/>
+    <col min="13" max="13" width="5.85546875" customWidth="1"/>
+    <col min="14" max="14" width="6.42578125" customWidth="1"/>
+    <col min="15" max="15" width="5.7109375" customWidth="1"/>
+    <col min="19" max="19" width="8.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="21"/>
-      <c r="C1" s="16" t="s">
+    <row r="1" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-    </row>
-    <row r="2" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="23" t="s">
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+    </row>
+    <row r="2" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="N3" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="S3" s="23" t="s">
+      <c r="S3" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="T3" s="17" t="s">
+      <c r="T3" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B4" s="24" t="s">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B4" s="16" t="s">
         <v>33</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1486,18 +1723,18 @@
       <c r="N4" s="6">
         <v>8</v>
       </c>
-      <c r="O4" s="10">
+      <c r="O4" s="2">
         <v>7</v>
       </c>
-      <c r="S4" s="24" t="s">
+      <c r="S4" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="T4" s="18">
+      <c r="T4" s="9">
         <v>1876</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B5" s="25"/>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B5" s="17"/>
       <c r="C5" s="3" t="s">
         <v>44</v>
       </c>
@@ -1532,18 +1769,18 @@
       <c r="N5" s="5">
         <v>3</v>
       </c>
-      <c r="O5" s="11">
-        <v>4</v>
-      </c>
-      <c r="S5" s="24" t="s">
+      <c r="O5" s="4">
+        <v>4</v>
+      </c>
+      <c r="S5" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="T5" s="19">
+      <c r="T5" s="10">
         <v>2190</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B6" s="24"/>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B6" s="16"/>
       <c r="C6" s="1" t="s">
         <v>39</v>
       </c>
@@ -1580,18 +1817,18 @@
       <c r="N6" s="6">
         <v>4</v>
       </c>
-      <c r="O6" s="10">
-        <v>1</v>
-      </c>
-      <c r="S6" s="24" t="s">
+      <c r="O6" s="2">
+        <v>1</v>
+      </c>
+      <c r="S6" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="T6" s="18">
+      <c r="T6" s="9">
         <v>3099</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B7" s="25"/>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B7" s="17"/>
       <c r="C7" s="3" t="s">
         <v>49</v>
       </c>
@@ -1612,18 +1849,18 @@
         <v>1</v>
       </c>
       <c r="N7" s="5"/>
-      <c r="O7" s="11">
-        <v>1</v>
-      </c>
-      <c r="S7" s="24" t="s">
+      <c r="O7" s="4">
+        <v>1</v>
+      </c>
+      <c r="S7" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="T7" s="19">
+      <c r="T7" s="10">
         <v>2793</v>
       </c>
     </row>
-    <row r="8" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="24"/>
+    <row r="8" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="16"/>
       <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
@@ -1640,16 +1877,16 @@
       <c r="L8" s="6"/>
       <c r="M8" s="2"/>
       <c r="N8" s="6"/>
-      <c r="O8" s="10"/>
-      <c r="S8" s="28" t="s">
+      <c r="O8" s="2"/>
+      <c r="S8" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="T8" s="20">
+      <c r="T8" s="11">
         <v>2484</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B9" s="25"/>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B9" s="17"/>
       <c r="C9" s="3" t="s">
         <v>41</v>
       </c>
@@ -1686,12 +1923,12 @@
       <c r="N9" s="5">
         <v>1</v>
       </c>
-      <c r="O9" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B10" s="24"/>
+      <c r="O9" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B10" s="16"/>
       <c r="C10" s="1" t="s">
         <v>46</v>
       </c>
@@ -1708,10 +1945,10 @@
       <c r="L10" s="6"/>
       <c r="M10" s="2"/>
       <c r="N10" s="6"/>
-      <c r="O10" s="10"/>
-    </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B11" s="25"/>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B11" s="17"/>
       <c r="C11" s="3" t="s">
         <v>40</v>
       </c>
@@ -1748,12 +1985,12 @@
       <c r="N11" s="5">
         <v>6</v>
       </c>
-      <c r="O11" s="11">
+      <c r="O11" s="4">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B12" s="24"/>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B12" s="16"/>
       <c r="C12" s="1" t="s">
         <v>5</v>
       </c>
@@ -1788,12 +2025,12 @@
       <c r="N12" s="6">
         <v>5</v>
       </c>
-      <c r="O12" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B13" s="25"/>
+      <c r="O12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B13" s="17"/>
       <c r="C13" s="3" t="s">
         <v>0</v>
       </c>
@@ -1830,12 +2067,12 @@
       <c r="N13" s="5">
         <v>22</v>
       </c>
-      <c r="O13" s="11">
+      <c r="O13" s="4">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B14" s="24"/>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B14" s="16"/>
       <c r="C14" s="1" t="s">
         <v>42</v>
       </c>
@@ -1872,12 +2109,12 @@
       <c r="N14" s="6">
         <v>4</v>
       </c>
-      <c r="O14" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B15" s="25"/>
+      <c r="O14" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B15" s="17"/>
       <c r="C15" s="3" t="s">
         <v>16</v>
       </c>
@@ -1896,12 +2133,12 @@
       <c r="N15" s="5">
         <v>1</v>
       </c>
-      <c r="O15" s="11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B16" s="24"/>
+      <c r="O15" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B16" s="16"/>
       <c r="C16" s="1" t="s">
         <v>13</v>
       </c>
@@ -1922,10 +2159,10 @@
         <v>1</v>
       </c>
       <c r="N16" s="6"/>
-      <c r="O16" s="10"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B17" s="25"/>
+      <c r="O16" s="2"/>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B17" s="17"/>
       <c r="C17" s="3" t="s">
         <v>9</v>
       </c>
@@ -1950,10 +2187,10 @@
       <c r="N17" s="5">
         <v>1</v>
       </c>
-      <c r="O17" s="11"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B18" s="24"/>
+      <c r="O17" s="4"/>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B18" s="16"/>
       <c r="C18" s="1" t="s">
         <v>4</v>
       </c>
@@ -1970,10 +2207,10 @@
       <c r="L18" s="6"/>
       <c r="M18" s="2"/>
       <c r="N18" s="6"/>
-      <c r="O18" s="10"/>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B19" s="25"/>
+      <c r="O18" s="2"/>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B19" s="17"/>
       <c r="C19" s="3" t="s">
         <v>14</v>
       </c>
@@ -1994,10 +2231,10 @@
         <v>1</v>
       </c>
       <c r="N19" s="5"/>
-      <c r="O19" s="11"/>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B20" s="24"/>
+      <c r="O19" s="4"/>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B20" s="16"/>
       <c r="C20" s="1" t="s">
         <v>19</v>
       </c>
@@ -2016,10 +2253,10 @@
         <v>1</v>
       </c>
       <c r="N20" s="6"/>
-      <c r="O20" s="10"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B21" s="25"/>
+      <c r="O20" s="2"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B21" s="17"/>
       <c r="C21" s="3" t="s">
         <v>11</v>
       </c>
@@ -2038,10 +2275,10 @@
         <v>1</v>
       </c>
       <c r="N21" s="5"/>
-      <c r="O21" s="11"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B22" s="24"/>
+      <c r="O21" s="4"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B22" s="16"/>
       <c r="C22" s="1" t="s">
         <v>8</v>
       </c>
@@ -2060,10 +2297,10 @@
       <c r="L22" s="6"/>
       <c r="M22" s="2"/>
       <c r="N22" s="6"/>
-      <c r="O22" s="10"/>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="25"/>
+      <c r="O22" s="2"/>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B23" s="17"/>
       <c r="C23" s="3" t="s">
         <v>20</v>
       </c>
@@ -2100,12 +2337,12 @@
       <c r="N23" s="5">
         <v>10</v>
       </c>
-      <c r="O23" s="11">
+      <c r="O23" s="4">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B24" s="24"/>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B24" s="16"/>
       <c r="C24" s="1" t="s">
         <v>50</v>
       </c>
@@ -2132,12 +2369,12 @@
         <v>1</v>
       </c>
       <c r="N24" s="6"/>
-      <c r="O24" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B25" s="25"/>
+      <c r="O24" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B25" s="17"/>
       <c r="C25" s="3" t="s">
         <v>3</v>
       </c>
@@ -2158,12 +2395,12 @@
       <c r="N25" s="5">
         <v>2</v>
       </c>
-      <c r="O25" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="24"/>
+      <c r="O25" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B26" s="16"/>
       <c r="C26" s="1" t="s">
         <v>18</v>
       </c>
@@ -2200,12 +2437,12 @@
       <c r="N26" s="6">
         <v>3</v>
       </c>
-      <c r="O26" s="10">
+      <c r="O26" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B27" s="25"/>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B27" s="17"/>
       <c r="C27" s="3" t="s">
         <v>45</v>
       </c>
@@ -2242,12 +2479,12 @@
       <c r="N27" s="5">
         <v>10</v>
       </c>
-      <c r="O27" s="11">
+      <c r="O27" s="4">
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B28" s="24"/>
+    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B28" s="16"/>
       <c r="C28" s="1" t="s">
         <v>12</v>
       </c>
@@ -2270,12 +2507,12 @@
       </c>
       <c r="M28" s="2"/>
       <c r="N28" s="6"/>
-      <c r="O28" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B29" s="25"/>
+      <c r="O28" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B29" s="17"/>
       <c r="C29" s="3" t="s">
         <v>2</v>
       </c>
@@ -2312,12 +2549,12 @@
       <c r="N29" s="5">
         <v>4</v>
       </c>
-      <c r="O29" s="11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B30" s="24"/>
+      <c r="O29" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B30" s="16"/>
       <c r="C30" s="1" t="s">
         <v>38</v>
       </c>
@@ -2354,12 +2591,12 @@
       <c r="N30" s="6">
         <v>78</v>
       </c>
-      <c r="O30" s="10">
+      <c r="O30" s="2">
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B31" s="25"/>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B31" s="17"/>
       <c r="C31" s="3" t="s">
         <v>7</v>
       </c>
@@ -2378,10 +2615,10 @@
         <v>1</v>
       </c>
       <c r="N31" s="5"/>
-      <c r="O31" s="11"/>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B32" s="24"/>
+      <c r="O31" s="4"/>
+    </row>
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B32" s="16"/>
       <c r="C32" s="1" t="s">
         <v>47</v>
       </c>
@@ -2404,12 +2641,12 @@
         <v>1</v>
       </c>
       <c r="N32" s="6"/>
-      <c r="O32" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B33" s="25"/>
+      <c r="O32" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B33" s="17"/>
       <c r="C33" s="3" t="s">
         <v>6</v>
       </c>
@@ -2436,10 +2673,10 @@
       <c r="N33" s="5">
         <v>2</v>
       </c>
-      <c r="O33" s="11"/>
-    </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B34" s="26"/>
+      <c r="O33" s="4"/>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B34" s="18"/>
       <c r="C34" s="1" t="s">
         <v>48</v>
       </c>
@@ -2466,12 +2703,12 @@
       <c r="N34" s="6">
         <v>1</v>
       </c>
-      <c r="O34" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B35" s="25" t="s">
+      <c r="O34" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B35" s="17" t="s">
         <v>34</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -2510,12 +2747,12 @@
       <c r="N35" s="5">
         <v>6</v>
       </c>
-      <c r="O35" s="11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B36" s="24"/>
+      <c r="O35" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B36" s="16"/>
       <c r="C36" s="1" t="s">
         <v>44</v>
       </c>
@@ -2552,12 +2789,12 @@
       <c r="N36" s="6">
         <v>2</v>
       </c>
-      <c r="O36" s="10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B37" s="25"/>
+      <c r="O36" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B37" s="17"/>
       <c r="C37" s="3" t="s">
         <v>39</v>
       </c>
@@ -2594,12 +2831,12 @@
       <c r="N37" s="5">
         <v>14</v>
       </c>
-      <c r="O37" s="11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B38" s="24"/>
+      <c r="O37" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B38" s="16"/>
       <c r="C38" s="1" t="s">
         <v>49</v>
       </c>
@@ -2616,10 +2853,10 @@
       </c>
       <c r="M38" s="2"/>
       <c r="N38" s="6"/>
-      <c r="O38" s="10"/>
-    </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B39" s="25"/>
+      <c r="O38" s="2"/>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B39" s="17"/>
       <c r="C39" s="3" t="s">
         <v>10</v>
       </c>
@@ -2638,10 +2875,10 @@
       </c>
       <c r="M39" s="4"/>
       <c r="N39" s="5"/>
-      <c r="O39" s="11"/>
-    </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B40" s="24"/>
+      <c r="O39" s="4"/>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B40" s="16"/>
       <c r="C40" s="1" t="s">
         <v>41</v>
       </c>
@@ -2676,10 +2913,10 @@
         <v>4</v>
       </c>
       <c r="N40" s="6"/>
-      <c r="O40" s="10"/>
-    </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B41" s="25"/>
+      <c r="O40" s="2"/>
+    </row>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B41" s="17"/>
       <c r="C41" s="3" t="s">
         <v>46</v>
       </c>
@@ -2698,12 +2935,12 @@
       <c r="L41" s="5"/>
       <c r="M41" s="4"/>
       <c r="N41" s="5"/>
-      <c r="O41" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B42" s="24"/>
+      <c r="O41" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B42" s="16"/>
       <c r="C42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2740,12 +2977,12 @@
       <c r="N42" s="6">
         <v>11</v>
       </c>
-      <c r="O42" s="10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B43" s="25"/>
+      <c r="O42" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B43" s="17"/>
       <c r="C43" s="3" t="s">
         <v>5</v>
       </c>
@@ -2782,10 +3019,10 @@
       <c r="N43" s="5">
         <v>3</v>
       </c>
-      <c r="O43" s="11"/>
-    </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B44" s="24"/>
+      <c r="O43" s="4"/>
+    </row>
+    <row r="44" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B44" s="16"/>
       <c r="C44" s="1" t="s">
         <v>0</v>
       </c>
@@ -2822,12 +3059,12 @@
       <c r="N44" s="6">
         <v>34</v>
       </c>
-      <c r="O44" s="10">
+      <c r="O44" s="2">
         <v>37</v>
       </c>
     </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B45" s="25"/>
+    <row r="45" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B45" s="17"/>
       <c r="C45" s="3" t="s">
         <v>42</v>
       </c>
@@ -2864,12 +3101,12 @@
       <c r="N45" s="5">
         <v>2</v>
       </c>
-      <c r="O45" s="11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B46" s="24"/>
+      <c r="O45" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B46" s="16"/>
       <c r="C46" s="1" t="s">
         <v>1</v>
       </c>
@@ -2888,10 +3125,10 @@
         <v>1</v>
       </c>
       <c r="N46" s="6"/>
-      <c r="O46" s="10"/>
-    </row>
-    <row r="47" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B47" s="25"/>
+      <c r="O46" s="2"/>
+    </row>
+    <row r="47" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B47" s="17"/>
       <c r="C47" s="3" t="s">
         <v>13</v>
       </c>
@@ -2910,12 +3147,12 @@
       <c r="L47" s="5"/>
       <c r="M47" s="4"/>
       <c r="N47" s="5"/>
-      <c r="O47" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B48" s="24"/>
+      <c r="O47" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B48" s="16"/>
       <c r="C48" s="1" t="s">
         <v>9</v>
       </c>
@@ -2944,12 +3181,12 @@
       <c r="N48" s="6">
         <v>2</v>
       </c>
-      <c r="O48" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B49" s="25"/>
+      <c r="O48" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B49" s="17"/>
       <c r="C49" s="3" t="s">
         <v>14</v>
       </c>
@@ -2976,12 +3213,12 @@
       <c r="N49" s="5">
         <v>1</v>
       </c>
-      <c r="O49" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B50" s="24"/>
+      <c r="O49" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B50" s="16"/>
       <c r="C50" s="1" t="s">
         <v>11</v>
       </c>
@@ -2998,10 +3235,10 @@
       <c r="L50" s="6"/>
       <c r="M50" s="2"/>
       <c r="N50" s="6"/>
-      <c r="O50" s="10"/>
-    </row>
-    <row r="51" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B51" s="25"/>
+      <c r="O50" s="2"/>
+    </row>
+    <row r="51" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B51" s="17"/>
       <c r="C51" s="3" t="s">
         <v>8</v>
       </c>
@@ -3022,10 +3259,10 @@
         <v>1</v>
       </c>
       <c r="N51" s="5"/>
-      <c r="O51" s="11"/>
-    </row>
-    <row r="52" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B52" s="24"/>
+      <c r="O51" s="4"/>
+    </row>
+    <row r="52" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B52" s="16"/>
       <c r="C52" s="1" t="s">
         <v>20</v>
       </c>
@@ -3062,12 +3299,12 @@
       <c r="N52" s="6">
         <v>20</v>
       </c>
-      <c r="O52" s="10">
+      <c r="O52" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="53" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B53" s="25"/>
+    <row r="53" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B53" s="17"/>
       <c r="C53" s="3" t="s">
         <v>50</v>
       </c>
@@ -3088,10 +3325,10 @@
       <c r="L53" s="5"/>
       <c r="M53" s="4"/>
       <c r="N53" s="5"/>
-      <c r="O53" s="11"/>
-    </row>
-    <row r="54" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B54" s="24"/>
+      <c r="O53" s="4"/>
+    </row>
+    <row r="54" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B54" s="16"/>
       <c r="C54" s="1" t="s">
         <v>3</v>
       </c>
@@ -3114,12 +3351,12 @@
         <v>2</v>
       </c>
       <c r="N54" s="6"/>
-      <c r="O54" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B55" s="25"/>
+      <c r="O54" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B55" s="17"/>
       <c r="C55" s="3" t="s">
         <v>18</v>
       </c>
@@ -3156,12 +3393,12 @@
       <c r="N55" s="5">
         <v>6</v>
       </c>
-      <c r="O55" s="11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="56" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B56" s="24"/>
+      <c r="O55" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B56" s="16"/>
       <c r="C56" s="1" t="s">
         <v>45</v>
       </c>
@@ -3198,12 +3435,12 @@
       <c r="N56" s="6">
         <v>6</v>
       </c>
-      <c r="O56" s="10">
+      <c r="O56" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B57" s="25"/>
+    <row r="57" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B57" s="17"/>
       <c r="C57" s="3" t="s">
         <v>12</v>
       </c>
@@ -3226,12 +3463,12 @@
       <c r="N57" s="5">
         <v>1</v>
       </c>
-      <c r="O57" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B58" s="24"/>
+      <c r="O57" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B58" s="16"/>
       <c r="C58" s="1" t="s">
         <v>2</v>
       </c>
@@ -3264,12 +3501,12 @@
       <c r="N58" s="6">
         <v>4</v>
       </c>
-      <c r="O58" s="10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="59" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B59" s="25"/>
+      <c r="O58" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B59" s="17"/>
       <c r="C59" s="3" t="s">
         <v>38</v>
       </c>
@@ -3306,12 +3543,12 @@
       <c r="N59" s="5">
         <v>79</v>
       </c>
-      <c r="O59" s="11">
+      <c r="O59" s="4">
         <v>76</v>
       </c>
     </row>
-    <row r="60" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B60" s="24"/>
+    <row r="60" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B60" s="16"/>
       <c r="C60" s="1" t="s">
         <v>7</v>
       </c>
@@ -3334,10 +3571,10 @@
       </c>
       <c r="M60" s="2"/>
       <c r="N60" s="6"/>
-      <c r="O60" s="10"/>
-    </row>
-    <row r="61" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B61" s="25"/>
+      <c r="O60" s="2"/>
+    </row>
+    <row r="61" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B61" s="17"/>
       <c r="C61" s="3" t="s">
         <v>47</v>
       </c>
@@ -3368,12 +3605,12 @@
       <c r="N61" s="5">
         <v>1</v>
       </c>
-      <c r="O61" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B62" s="24"/>
+      <c r="O61" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B62" s="16"/>
       <c r="C62" s="1" t="s">
         <v>6</v>
       </c>
@@ -3398,10 +3635,10 @@
       </c>
       <c r="M62" s="2"/>
       <c r="N62" s="6"/>
-      <c r="O62" s="10"/>
-    </row>
-    <row r="63" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B63" s="27"/>
+      <c r="O62" s="2"/>
+    </row>
+    <row r="63" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B63" s="19"/>
       <c r="C63" s="3" t="s">
         <v>48</v>
       </c>
@@ -3420,12 +3657,12 @@
       <c r="L63" s="5"/>
       <c r="M63" s="4"/>
       <c r="N63" s="5"/>
-      <c r="O63" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="24" t="s">
+      <c r="O63" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B64" s="16" t="s">
         <v>35</v>
       </c>
       <c r="C64" s="1" t="s">
@@ -3464,12 +3701,12 @@
       <c r="N64" s="6">
         <v>15</v>
       </c>
-      <c r="O64" s="10">
+      <c r="O64" s="2">
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="25"/>
+    <row r="65" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B65" s="17"/>
       <c r="C65" s="3" t="s">
         <v>44</v>
       </c>
@@ -3506,12 +3743,12 @@
       <c r="N65" s="5">
         <v>7</v>
       </c>
-      <c r="O65" s="11">
+      <c r="O65" s="4">
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="24"/>
+    <row r="66" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B66" s="16"/>
       <c r="C66" s="1" t="s">
         <v>39</v>
       </c>
@@ -3548,12 +3785,12 @@
       <c r="N66" s="6">
         <v>13</v>
       </c>
-      <c r="O66" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="67" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B67" s="25"/>
+      <c r="O66" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B67" s="17"/>
       <c r="C67" s="3" t="s">
         <v>49</v>
       </c>
@@ -3568,12 +3805,12 @@
       <c r="L67" s="5"/>
       <c r="M67" s="4"/>
       <c r="N67" s="5"/>
-      <c r="O67" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B68" s="24"/>
+      <c r="O67" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B68" s="16"/>
       <c r="C68" s="1" t="s">
         <v>10</v>
       </c>
@@ -3594,12 +3831,12 @@
         <v>2</v>
       </c>
       <c r="N68" s="6"/>
-      <c r="O68" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B69" s="25"/>
+      <c r="O68" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B69" s="17"/>
       <c r="C69" s="3" t="s">
         <v>41</v>
       </c>
@@ -3632,12 +3869,12 @@
       <c r="N69" s="5">
         <v>2</v>
       </c>
-      <c r="O69" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B70" s="24"/>
+      <c r="O69" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B70" s="16"/>
       <c r="C70" s="1" t="s">
         <v>46</v>
       </c>
@@ -3658,10 +3895,10 @@
       <c r="N70" s="6">
         <v>2</v>
       </c>
-      <c r="O70" s="10"/>
-    </row>
-    <row r="71" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B71" s="25"/>
+      <c r="O70" s="2"/>
+    </row>
+    <row r="71" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B71" s="17"/>
       <c r="C71" s="3" t="s">
         <v>40</v>
       </c>
@@ -3698,12 +3935,12 @@
       <c r="N71" s="5">
         <v>10</v>
       </c>
-      <c r="O71" s="11">
+      <c r="O71" s="4">
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B72" s="24"/>
+    <row r="72" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B72" s="16"/>
       <c r="C72" s="1" t="s">
         <v>5</v>
       </c>
@@ -3738,12 +3975,12 @@
       <c r="N72" s="6">
         <v>3</v>
       </c>
-      <c r="O72" s="10">
+      <c r="O72" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B73" s="25"/>
+    <row r="73" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B73" s="17"/>
       <c r="C73" s="3" t="s">
         <v>0</v>
       </c>
@@ -3780,12 +4017,12 @@
       <c r="N73" s="5">
         <v>42</v>
       </c>
-      <c r="O73" s="11">
+      <c r="O73" s="4">
         <v>40</v>
       </c>
     </row>
-    <row r="74" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B74" s="24"/>
+    <row r="74" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B74" s="16"/>
       <c r="C74" s="1" t="s">
         <v>42</v>
       </c>
@@ -3820,12 +4057,12 @@
       <c r="N74" s="6">
         <v>4</v>
       </c>
-      <c r="O74" s="10">
+      <c r="O74" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B75" s="25"/>
+    <row r="75" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B75" s="17"/>
       <c r="C75" s="3" t="s">
         <v>1</v>
       </c>
@@ -3850,10 +4087,10 @@
       <c r="N75" s="5">
         <v>1</v>
       </c>
-      <c r="O75" s="11"/>
-    </row>
-    <row r="76" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B76" s="24"/>
+      <c r="O75" s="4"/>
+    </row>
+    <row r="76" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B76" s="16"/>
       <c r="C76" s="1" t="s">
         <v>16</v>
       </c>
@@ -3872,10 +4109,10 @@
       </c>
       <c r="M76" s="2"/>
       <c r="N76" s="6"/>
-      <c r="O76" s="10"/>
-    </row>
-    <row r="77" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B77" s="25"/>
+      <c r="O76" s="2"/>
+    </row>
+    <row r="77" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B77" s="17"/>
       <c r="C77" s="3" t="s">
         <v>13</v>
       </c>
@@ -3894,10 +4131,10 @@
       <c r="L77" s="5"/>
       <c r="M77" s="4"/>
       <c r="N77" s="5"/>
-      <c r="O77" s="11"/>
-    </row>
-    <row r="78" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B78" s="24"/>
+      <c r="O77" s="4"/>
+    </row>
+    <row r="78" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B78" s="16"/>
       <c r="C78" s="1" t="s">
         <v>9</v>
       </c>
@@ -3924,10 +4161,10 @@
         <v>3</v>
       </c>
       <c r="N78" s="6"/>
-      <c r="O78" s="10"/>
-    </row>
-    <row r="79" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B79" s="25"/>
+      <c r="O78" s="2"/>
+    </row>
+    <row r="79" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B79" s="17"/>
       <c r="C79" s="3" t="s">
         <v>4</v>
       </c>
@@ -3944,10 +4181,10 @@
       <c r="L79" s="5"/>
       <c r="M79" s="4"/>
       <c r="N79" s="5"/>
-      <c r="O79" s="11"/>
-    </row>
-    <row r="80" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B80" s="24"/>
+      <c r="O79" s="4"/>
+    </row>
+    <row r="80" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B80" s="16"/>
       <c r="C80" s="1" t="s">
         <v>14</v>
       </c>
@@ -3972,12 +4209,12 @@
       <c r="L80" s="6"/>
       <c r="M80" s="2"/>
       <c r="N80" s="6"/>
-      <c r="O80" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="81" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B81" s="25"/>
+      <c r="O80" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B81" s="17"/>
       <c r="C81" s="3" t="s">
         <v>19</v>
       </c>
@@ -3994,10 +4231,10 @@
       <c r="L81" s="5"/>
       <c r="M81" s="4"/>
       <c r="N81" s="5"/>
-      <c r="O81" s="11"/>
-    </row>
-    <row r="82" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B82" s="24"/>
+      <c r="O81" s="4"/>
+    </row>
+    <row r="82" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B82" s="16"/>
       <c r="C82" s="1" t="s">
         <v>11</v>
       </c>
@@ -4016,10 +4253,10 @@
       </c>
       <c r="M82" s="2"/>
       <c r="N82" s="6"/>
-      <c r="O82" s="10"/>
-    </row>
-    <row r="83" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B83" s="25"/>
+      <c r="O82" s="2"/>
+    </row>
+    <row r="83" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B83" s="17"/>
       <c r="C83" s="3" t="s">
         <v>51</v>
       </c>
@@ -4040,12 +4277,12 @@
       <c r="N83" s="5">
         <v>1</v>
       </c>
-      <c r="O83" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B84" s="24"/>
+      <c r="O83" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B84" s="16"/>
       <c r="C84" s="1" t="s">
         <v>8</v>
       </c>
@@ -4068,10 +4305,10 @@
       <c r="N84" s="6">
         <v>2</v>
       </c>
-      <c r="O84" s="10"/>
-    </row>
-    <row r="85" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B85" s="25"/>
+      <c r="O84" s="2"/>
+    </row>
+    <row r="85" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B85" s="17"/>
       <c r="C85" s="3" t="s">
         <v>20</v>
       </c>
@@ -4108,12 +4345,12 @@
       <c r="N85" s="5">
         <v>23</v>
       </c>
-      <c r="O85" s="11">
+      <c r="O85" s="4">
         <v>22</v>
       </c>
     </row>
-    <row r="86" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B86" s="24"/>
+    <row r="86" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B86" s="16"/>
       <c r="C86" s="1" t="s">
         <v>50</v>
       </c>
@@ -4138,10 +4375,10 @@
         <v>1</v>
       </c>
       <c r="N86" s="6"/>
-      <c r="O86" s="10"/>
-    </row>
-    <row r="87" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B87" s="25"/>
+      <c r="O86" s="2"/>
+    </row>
+    <row r="87" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B87" s="17"/>
       <c r="C87" s="3" t="s">
         <v>3</v>
       </c>
@@ -4166,12 +4403,12 @@
         <v>2</v>
       </c>
       <c r="N87" s="5"/>
-      <c r="O87" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="88" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B88" s="24"/>
+      <c r="O87" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B88" s="16"/>
       <c r="C88" s="1" t="s">
         <v>18</v>
       </c>
@@ -4208,12 +4445,12 @@
       <c r="N88" s="6">
         <v>7</v>
       </c>
-      <c r="O88" s="10">
+      <c r="O88" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B89" s="25"/>
+    <row r="89" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B89" s="17"/>
       <c r="C89" s="3" t="s">
         <v>45</v>
       </c>
@@ -4250,12 +4487,12 @@
       <c r="N89" s="5">
         <v>7</v>
       </c>
-      <c r="O89" s="11">
+      <c r="O89" s="4">
         <v>8</v>
       </c>
     </row>
-    <row r="90" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B90" s="24"/>
+    <row r="90" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B90" s="16"/>
       <c r="C90" s="1" t="s">
         <v>12</v>
       </c>
@@ -4284,12 +4521,12 @@
         <v>3</v>
       </c>
       <c r="N90" s="6"/>
-      <c r="O90" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B91" s="25"/>
+      <c r="O90" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B91" s="17"/>
       <c r="C91" s="3" t="s">
         <v>2</v>
       </c>
@@ -4322,12 +4559,12 @@
         <v>6</v>
       </c>
       <c r="N91" s="5"/>
-      <c r="O91" s="11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="92" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B92" s="24"/>
+      <c r="O91" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B92" s="16"/>
       <c r="C92" s="1" t="s">
         <v>15</v>
       </c>
@@ -4348,12 +4585,12 @@
       <c r="N92" s="6">
         <v>3</v>
       </c>
-      <c r="O92" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B93" s="25"/>
+      <c r="O92" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B93" s="17"/>
       <c r="C93" s="3" t="s">
         <v>38</v>
       </c>
@@ -4390,12 +4627,12 @@
       <c r="N93" s="5">
         <v>97</v>
       </c>
-      <c r="O93" s="11">
+      <c r="O93" s="4">
         <v>135</v>
       </c>
     </row>
-    <row r="94" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B94" s="24"/>
+    <row r="94" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B94" s="16"/>
       <c r="C94" s="1" t="s">
         <v>7</v>
       </c>
@@ -4426,10 +4663,10 @@
         <v>1</v>
       </c>
       <c r="N94" s="6"/>
-      <c r="O94" s="10"/>
-    </row>
-    <row r="95" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B95" s="25"/>
+      <c r="O94" s="2"/>
+    </row>
+    <row r="95" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B95" s="17"/>
       <c r="C95" s="3" t="s">
         <v>47</v>
       </c>
@@ -4464,12 +4701,12 @@
       <c r="N95" s="5">
         <v>2</v>
       </c>
-      <c r="O95" s="11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="96" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B96" s="24"/>
+      <c r="O95" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="96" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B96" s="16"/>
       <c r="C96" s="1" t="s">
         <v>6</v>
       </c>
@@ -4498,12 +4735,12 @@
         <v>1</v>
       </c>
       <c r="N96" s="6"/>
-      <c r="O96" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="97" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B97" s="27"/>
+      <c r="O96" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B97" s="19"/>
       <c r="C97" s="3" t="s">
         <v>48</v>
       </c>
@@ -4536,10 +4773,10 @@
       <c r="N97" s="5">
         <v>2</v>
       </c>
-      <c r="O97" s="11"/>
-    </row>
-    <row r="98" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B98" s="24" t="s">
+      <c r="O97" s="4"/>
+    </row>
+    <row r="98" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B98" s="16" t="s">
         <v>36</v>
       </c>
       <c r="C98" s="1" t="s">
@@ -4578,12 +4815,12 @@
       <c r="N98" s="6">
         <v>8</v>
       </c>
-      <c r="O98" s="10">
+      <c r="O98" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B99" s="25"/>
+    <row r="99" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B99" s="17"/>
       <c r="C99" s="3" t="s">
         <v>44</v>
       </c>
@@ -4620,12 +4857,12 @@
       <c r="N99" s="5">
         <v>3</v>
       </c>
-      <c r="O99" s="11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="100" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B100" s="24"/>
+      <c r="O99" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B100" s="16"/>
       <c r="C100" s="1" t="s">
         <v>39</v>
       </c>
@@ -4662,12 +4899,12 @@
       <c r="N100" s="6">
         <v>9</v>
       </c>
-      <c r="O100" s="10">
+      <c r="O100" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B101" s="25"/>
+    <row r="101" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B101" s="17"/>
       <c r="C101" s="3" t="s">
         <v>49</v>
       </c>
@@ -4686,10 +4923,10 @@
       <c r="L101" s="5"/>
       <c r="M101" s="4"/>
       <c r="N101" s="5"/>
-      <c r="O101" s="11"/>
-    </row>
-    <row r="102" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B102" s="24"/>
+      <c r="O101" s="4"/>
+    </row>
+    <row r="102" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B102" s="16"/>
       <c r="C102" s="1" t="s">
         <v>10</v>
       </c>
@@ -4708,10 +4945,10 @@
       <c r="L102" s="6"/>
       <c r="M102" s="2"/>
       <c r="N102" s="6"/>
-      <c r="O102" s="10"/>
-    </row>
-    <row r="103" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B103" s="25"/>
+      <c r="O102" s="2"/>
+    </row>
+    <row r="103" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B103" s="17"/>
       <c r="C103" s="3" t="s">
         <v>41</v>
       </c>
@@ -4744,10 +4981,10 @@
       <c r="N103" s="5">
         <v>4</v>
       </c>
-      <c r="O103" s="11"/>
-    </row>
-    <row r="104" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B104" s="24"/>
+      <c r="O103" s="4"/>
+    </row>
+    <row r="104" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B104" s="16"/>
       <c r="C104" s="1" t="s">
         <v>46</v>
       </c>
@@ -4768,10 +5005,10 @@
       <c r="N104" s="6">
         <v>1</v>
       </c>
-      <c r="O104" s="10"/>
-    </row>
-    <row r="105" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B105" s="25"/>
+      <c r="O104" s="2"/>
+    </row>
+    <row r="105" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B105" s="17"/>
       <c r="C105" s="3" t="s">
         <v>40</v>
       </c>
@@ -4808,12 +5045,12 @@
       <c r="N105" s="5">
         <v>4</v>
       </c>
-      <c r="O105" s="11">
+      <c r="O105" s="4">
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B106" s="24"/>
+    <row r="106" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B106" s="16"/>
       <c r="C106" s="1" t="s">
         <v>5</v>
       </c>
@@ -4850,12 +5087,12 @@
       <c r="N106" s="6">
         <v>9</v>
       </c>
-      <c r="O106" s="10">
+      <c r="O106" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B107" s="25"/>
+    <row r="107" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B107" s="17"/>
       <c r="C107" s="3" t="s">
         <v>0</v>
       </c>
@@ -4892,12 +5129,12 @@
       <c r="N107" s="5">
         <v>32</v>
       </c>
-      <c r="O107" s="11">
+      <c r="O107" s="4">
         <v>53</v>
       </c>
     </row>
-    <row r="108" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B108" s="24"/>
+    <row r="108" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B108" s="16"/>
       <c r="C108" s="1" t="s">
         <v>42</v>
       </c>
@@ -4930,10 +5167,10 @@
       <c r="N108" s="6">
         <v>2</v>
       </c>
-      <c r="O108" s="10"/>
-    </row>
-    <row r="109" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B109" s="25"/>
+      <c r="O108" s="2"/>
+    </row>
+    <row r="109" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B109" s="17"/>
       <c r="C109" s="3" t="s">
         <v>1</v>
       </c>
@@ -4962,12 +5199,12 @@
       <c r="N109" s="5">
         <v>1</v>
       </c>
-      <c r="O109" s="11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="110" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B110" s="24"/>
+      <c r="O109" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B110" s="16"/>
       <c r="C110" s="1" t="s">
         <v>16</v>
       </c>
@@ -4990,10 +5227,10 @@
       <c r="L110" s="6"/>
       <c r="M110" s="2"/>
       <c r="N110" s="6"/>
-      <c r="O110" s="10"/>
-    </row>
-    <row r="111" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B111" s="25"/>
+      <c r="O110" s="2"/>
+    </row>
+    <row r="111" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B111" s="17"/>
       <c r="C111" s="3" t="s">
         <v>13</v>
       </c>
@@ -5012,10 +5249,10 @@
       <c r="L111" s="5"/>
       <c r="M111" s="4"/>
       <c r="N111" s="5"/>
-      <c r="O111" s="11"/>
-    </row>
-    <row r="112" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B112" s="24"/>
+      <c r="O111" s="4"/>
+    </row>
+    <row r="112" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B112" s="16"/>
       <c r="C112" s="1" t="s">
         <v>9</v>
       </c>
@@ -5042,12 +5279,12 @@
       </c>
       <c r="M112" s="2"/>
       <c r="N112" s="6"/>
-      <c r="O112" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="113" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B113" s="25"/>
+      <c r="O112" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B113" s="17"/>
       <c r="C113" s="3" t="s">
         <v>4</v>
       </c>
@@ -5064,10 +5301,10 @@
       <c r="N113" s="5">
         <v>1</v>
       </c>
-      <c r="O113" s="11"/>
-    </row>
-    <row r="114" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B114" s="24"/>
+      <c r="O113" s="4"/>
+    </row>
+    <row r="114" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B114" s="16"/>
       <c r="C114" s="1" t="s">
         <v>14</v>
       </c>
@@ -5088,10 +5325,10 @@
       <c r="N114" s="6">
         <v>1</v>
       </c>
-      <c r="O114" s="10"/>
-    </row>
-    <row r="115" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B115" s="25"/>
+      <c r="O114" s="2"/>
+    </row>
+    <row r="115" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B115" s="17"/>
       <c r="C115" s="3" t="s">
         <v>11</v>
       </c>
@@ -5108,10 +5345,10 @@
       <c r="L115" s="5"/>
       <c r="M115" s="4"/>
       <c r="N115" s="5"/>
-      <c r="O115" s="11"/>
-    </row>
-    <row r="116" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B116" s="24"/>
+      <c r="O115" s="4"/>
+    </row>
+    <row r="116" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B116" s="16"/>
       <c r="C116" s="1" t="s">
         <v>51</v>
       </c>
@@ -5128,10 +5365,10 @@
       <c r="L116" s="6"/>
       <c r="M116" s="2"/>
       <c r="N116" s="6"/>
-      <c r="O116" s="10"/>
-    </row>
-    <row r="117" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B117" s="25"/>
+      <c r="O116" s="2"/>
+    </row>
+    <row r="117" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B117" s="17"/>
       <c r="C117" s="3" t="s">
         <v>8</v>
       </c>
@@ -5156,12 +5393,12 @@
         <v>1</v>
       </c>
       <c r="N117" s="5"/>
-      <c r="O117" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="118" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B118" s="24"/>
+      <c r="O117" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B118" s="16"/>
       <c r="C118" s="1" t="s">
         <v>20</v>
       </c>
@@ -5198,12 +5435,12 @@
       <c r="N118" s="6">
         <v>23</v>
       </c>
-      <c r="O118" s="10">
+      <c r="O118" s="2">
         <v>14</v>
       </c>
     </row>
-    <row r="119" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B119" s="25"/>
+    <row r="119" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B119" s="17"/>
       <c r="C119" s="3" t="s">
         <v>50</v>
       </c>
@@ -5232,12 +5469,12 @@
       <c r="N119" s="5">
         <v>1</v>
       </c>
-      <c r="O119" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="120" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B120" s="24"/>
+      <c r="O119" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B120" s="16"/>
       <c r="C120" s="1" t="s">
         <v>3</v>
       </c>
@@ -5260,12 +5497,12 @@
       <c r="N120" s="6">
         <v>1</v>
       </c>
-      <c r="O120" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="121" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B121" s="25"/>
+      <c r="O120" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B121" s="17"/>
       <c r="C121" s="3" t="s">
         <v>18</v>
       </c>
@@ -5302,12 +5539,12 @@
       <c r="N121" s="5">
         <v>1</v>
       </c>
-      <c r="O121" s="11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="122" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B122" s="24"/>
+      <c r="O121" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="122" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B122" s="16"/>
       <c r="C122" s="1" t="s">
         <v>17</v>
       </c>
@@ -5324,10 +5561,10 @@
       <c r="L122" s="6"/>
       <c r="M122" s="2"/>
       <c r="N122" s="6"/>
-      <c r="O122" s="10"/>
-    </row>
-    <row r="123" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B123" s="25"/>
+      <c r="O122" s="2"/>
+    </row>
+    <row r="123" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B123" s="17"/>
       <c r="C123" s="3" t="s">
         <v>45</v>
       </c>
@@ -5364,12 +5601,12 @@
       <c r="N123" s="5">
         <v>14</v>
       </c>
-      <c r="O123" s="11">
+      <c r="O123" s="4">
         <v>21</v>
       </c>
     </row>
-    <row r="124" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B124" s="24"/>
+    <row r="124" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B124" s="16"/>
       <c r="C124" s="1" t="s">
         <v>12</v>
       </c>
@@ -5402,12 +5639,12 @@
       <c r="N124" s="6">
         <v>1</v>
       </c>
-      <c r="O124" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="125" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B125" s="25"/>
+      <c r="O124" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B125" s="17"/>
       <c r="C125" s="3" t="s">
         <v>2</v>
       </c>
@@ -5444,12 +5681,12 @@
       <c r="N125" s="5">
         <v>6</v>
       </c>
-      <c r="O125" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="126" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B126" s="24"/>
+      <c r="O125" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="126" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B126" s="16"/>
       <c r="C126" s="1" t="s">
         <v>15</v>
       </c>
@@ -5468,10 +5705,10 @@
         <v>1</v>
       </c>
       <c r="N126" s="6"/>
-      <c r="O126" s="10"/>
-    </row>
-    <row r="127" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B127" s="25"/>
+      <c r="O126" s="2"/>
+    </row>
+    <row r="127" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B127" s="17"/>
       <c r="C127" s="3" t="s">
         <v>38</v>
       </c>
@@ -5508,12 +5745,12 @@
       <c r="N127" s="5">
         <v>77</v>
       </c>
-      <c r="O127" s="11">
+      <c r="O127" s="4">
         <v>73</v>
       </c>
     </row>
-    <row r="128" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B128" s="24"/>
+    <row r="128" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B128" s="16"/>
       <c r="C128" s="1" t="s">
         <v>7</v>
       </c>
@@ -5538,12 +5775,12 @@
         <v>1</v>
       </c>
       <c r="N128" s="6"/>
-      <c r="O128" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="129" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B129" s="25"/>
+      <c r="O128" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B129" s="17"/>
       <c r="C129" s="3" t="s">
         <v>47</v>
       </c>
@@ -5576,10 +5813,10 @@
       <c r="N129" s="5">
         <v>2</v>
       </c>
-      <c r="O129" s="11"/>
-    </row>
-    <row r="130" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B130" s="24"/>
+      <c r="O129" s="4"/>
+    </row>
+    <row r="130" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B130" s="16"/>
       <c r="C130" s="1" t="s">
         <v>6</v>
       </c>
@@ -5612,12 +5849,12 @@
       <c r="N130" s="6">
         <v>1</v>
       </c>
-      <c r="O130" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="131" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B131" s="27"/>
+      <c r="O130" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B131" s="19"/>
       <c r="C131" s="3" t="s">
         <v>48</v>
       </c>
@@ -5638,12 +5875,12 @@
       <c r="L131" s="5"/>
       <c r="M131" s="4"/>
       <c r="N131" s="5"/>
-      <c r="O131" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="132" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B132" s="24" t="s">
+      <c r="O131" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B132" s="16" t="s">
         <v>37</v>
       </c>
       <c r="C132" s="1" t="s">
@@ -5682,12 +5919,12 @@
       <c r="N132" s="6">
         <v>15</v>
       </c>
-      <c r="O132" s="10">
+      <c r="O132" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="133" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B133" s="25"/>
+    <row r="133" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B133" s="17"/>
       <c r="C133" s="3" t="s">
         <v>44</v>
       </c>
@@ -5724,12 +5961,12 @@
       <c r="N133" s="5">
         <v>1</v>
       </c>
-      <c r="O133" s="11">
+      <c r="O133" s="4">
         <v>6</v>
       </c>
     </row>
-    <row r="134" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B134" s="24"/>
+    <row r="134" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B134" s="16"/>
       <c r="C134" s="1" t="s">
         <v>39</v>
       </c>
@@ -5766,12 +6003,12 @@
       <c r="N134" s="6">
         <v>8</v>
       </c>
-      <c r="O134" s="10">
+      <c r="O134" s="2">
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B135" s="25"/>
+    <row r="135" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B135" s="17"/>
       <c r="C135" s="3" t="s">
         <v>49</v>
       </c>
@@ -5796,10 +6033,10 @@
       <c r="N135" s="5">
         <v>1</v>
       </c>
-      <c r="O135" s="11"/>
-    </row>
-    <row r="136" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B136" s="24"/>
+      <c r="O135" s="4"/>
+    </row>
+    <row r="136" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B136" s="16"/>
       <c r="C136" s="1" t="s">
         <v>10</v>
       </c>
@@ -5820,10 +6057,10 @@
         <v>1</v>
       </c>
       <c r="N136" s="6"/>
-      <c r="O136" s="10"/>
-    </row>
-    <row r="137" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B137" s="25"/>
+      <c r="O136" s="2"/>
+    </row>
+    <row r="137" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B137" s="17"/>
       <c r="C137" s="3" t="s">
         <v>41</v>
       </c>
@@ -5856,12 +6093,12 @@
       <c r="N137" s="5">
         <v>4</v>
       </c>
-      <c r="O137" s="11">
+      <c r="O137" s="4">
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B138" s="24"/>
+    <row r="138" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B138" s="16"/>
       <c r="C138" s="1" t="s">
         <v>46</v>
       </c>
@@ -5886,10 +6123,10 @@
         <v>2</v>
       </c>
       <c r="N138" s="6"/>
-      <c r="O138" s="10"/>
-    </row>
-    <row r="139" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B139" s="25"/>
+      <c r="O138" s="2"/>
+    </row>
+    <row r="139" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B139" s="17"/>
       <c r="C139" s="3" t="s">
         <v>40</v>
       </c>
@@ -5926,12 +6163,12 @@
       <c r="N139" s="5">
         <v>15</v>
       </c>
-      <c r="O139" s="11">
+      <c r="O139" s="4">
         <v>8</v>
       </c>
     </row>
-    <row r="140" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B140" s="24"/>
+    <row r="140" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B140" s="16"/>
       <c r="C140" s="1" t="s">
         <v>5</v>
       </c>
@@ -5968,12 +6205,12 @@
       <c r="N140" s="6">
         <v>6</v>
       </c>
-      <c r="O140" s="10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="141" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B141" s="25"/>
+      <c r="O140" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="141" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B141" s="17"/>
       <c r="C141" s="3" t="s">
         <v>0</v>
       </c>
@@ -6010,12 +6247,12 @@
       <c r="N141" s="5">
         <v>29</v>
       </c>
-      <c r="O141" s="11">
+      <c r="O141" s="4">
         <v>20</v>
       </c>
     </row>
-    <row r="142" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B142" s="24"/>
+    <row r="142" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B142" s="16"/>
       <c r="C142" s="1" t="s">
         <v>42</v>
       </c>
@@ -6046,12 +6283,12 @@
         <v>5</v>
       </c>
       <c r="N142" s="6"/>
-      <c r="O142" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="143" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B143" s="25"/>
+      <c r="O142" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B143" s="17"/>
       <c r="C143" s="3" t="s">
         <v>1</v>
       </c>
@@ -6072,10 +6309,10 @@
       <c r="L143" s="5"/>
       <c r="M143" s="4"/>
       <c r="N143" s="5"/>
-      <c r="O143" s="11"/>
-    </row>
-    <row r="144" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B144" s="24"/>
+      <c r="O143" s="4"/>
+    </row>
+    <row r="144" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B144" s="16"/>
       <c r="C144" s="1" t="s">
         <v>16</v>
       </c>
@@ -6096,10 +6333,10 @@
       <c r="L144" s="6"/>
       <c r="M144" s="2"/>
       <c r="N144" s="6"/>
-      <c r="O144" s="10"/>
-    </row>
-    <row r="145" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B145" s="25"/>
+      <c r="O144" s="2"/>
+    </row>
+    <row r="145" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B145" s="17"/>
       <c r="C145" s="3" t="s">
         <v>13</v>
       </c>
@@ -6118,10 +6355,10 @@
         <v>2</v>
       </c>
       <c r="N145" s="5"/>
-      <c r="O145" s="11"/>
-    </row>
-    <row r="146" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B146" s="24"/>
+      <c r="O145" s="4"/>
+    </row>
+    <row r="146" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B146" s="16"/>
       <c r="C146" s="1" t="s">
         <v>9</v>
       </c>
@@ -6156,12 +6393,12 @@
       <c r="N146" s="6">
         <v>2</v>
       </c>
-      <c r="O146" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="147" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B147" s="25"/>
+      <c r="O146" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="147" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B147" s="17"/>
       <c r="C147" s="3" t="s">
         <v>14</v>
       </c>
@@ -6184,10 +6421,10 @@
       <c r="N147" s="5">
         <v>2</v>
       </c>
-      <c r="O147" s="11"/>
-    </row>
-    <row r="148" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B148" s="24"/>
+      <c r="O147" s="4"/>
+    </row>
+    <row r="148" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B148" s="16"/>
       <c r="C148" s="1" t="s">
         <v>19</v>
       </c>
@@ -6206,10 +6443,10 @@
       <c r="N148" s="6">
         <v>1</v>
       </c>
-      <c r="O148" s="10"/>
-    </row>
-    <row r="149" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B149" s="25"/>
+      <c r="O148" s="2"/>
+    </row>
+    <row r="149" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B149" s="17"/>
       <c r="C149" s="3" t="s">
         <v>11</v>
       </c>
@@ -6226,10 +6463,10 @@
       <c r="L149" s="5"/>
       <c r="M149" s="4"/>
       <c r="N149" s="5"/>
-      <c r="O149" s="11"/>
-    </row>
-    <row r="150" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B150" s="24"/>
+      <c r="O149" s="4"/>
+    </row>
+    <row r="150" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B150" s="16"/>
       <c r="C150" s="1" t="s">
         <v>51</v>
       </c>
@@ -6246,10 +6483,10 @@
       <c r="N150" s="6">
         <v>1</v>
       </c>
-      <c r="O150" s="10"/>
-    </row>
-    <row r="151" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B151" s="25"/>
+      <c r="O150" s="2"/>
+    </row>
+    <row r="151" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B151" s="17"/>
       <c r="C151" s="3" t="s">
         <v>8</v>
       </c>
@@ -6272,12 +6509,12 @@
       <c r="N151" s="5">
         <v>1</v>
       </c>
-      <c r="O151" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="152" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B152" s="24"/>
+      <c r="O151" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B152" s="16"/>
       <c r="C152" s="1" t="s">
         <v>20</v>
       </c>
@@ -6314,12 +6551,12 @@
       <c r="N152" s="6">
         <v>18</v>
       </c>
-      <c r="O152" s="10">
+      <c r="O152" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="153" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B153" s="25"/>
+    <row r="153" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B153" s="17"/>
       <c r="C153" s="3" t="s">
         <v>50</v>
       </c>
@@ -6338,10 +6575,10 @@
       <c r="L153" s="5"/>
       <c r="M153" s="4"/>
       <c r="N153" s="5"/>
-      <c r="O153" s="11"/>
-    </row>
-    <row r="154" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B154" s="24"/>
+      <c r="O153" s="4"/>
+    </row>
+    <row r="154" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B154" s="16"/>
       <c r="C154" s="1" t="s">
         <v>3</v>
       </c>
@@ -6362,12 +6599,12 @@
       <c r="L154" s="6"/>
       <c r="M154" s="2"/>
       <c r="N154" s="6"/>
-      <c r="O154" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="155" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B155" s="25"/>
+      <c r="O154" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B155" s="17"/>
       <c r="C155" s="3" t="s">
         <v>18</v>
       </c>
@@ -6404,12 +6641,12 @@
       <c r="N155" s="5">
         <v>2</v>
       </c>
-      <c r="O155" s="11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="156" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B156" s="24"/>
+      <c r="O155" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="156" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B156" s="16"/>
       <c r="C156" s="1" t="s">
         <v>45</v>
       </c>
@@ -6446,12 +6683,12 @@
       <c r="N156" s="6">
         <v>13</v>
       </c>
-      <c r="O156" s="10">
+      <c r="O156" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="157" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B157" s="25"/>
+    <row r="157" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B157" s="17"/>
       <c r="C157" s="3" t="s">
         <v>12</v>
       </c>
@@ -6478,10 +6715,10 @@
       </c>
       <c r="M157" s="4"/>
       <c r="N157" s="5"/>
-      <c r="O157" s="11"/>
-    </row>
-    <row r="158" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B158" s="24"/>
+      <c r="O157" s="4"/>
+    </row>
+    <row r="158" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B158" s="16"/>
       <c r="C158" s="1" t="s">
         <v>2</v>
       </c>
@@ -6518,12 +6755,12 @@
       <c r="N158" s="6">
         <v>2</v>
       </c>
-      <c r="O158" s="10">
+      <c r="O158" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="159" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B159" s="25"/>
+    <row r="159" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B159" s="17"/>
       <c r="C159" s="3" t="s">
         <v>15</v>
       </c>
@@ -6540,10 +6777,10 @@
       <c r="L159" s="5"/>
       <c r="M159" s="4"/>
       <c r="N159" s="5"/>
-      <c r="O159" s="11"/>
-    </row>
-    <row r="160" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B160" s="24"/>
+      <c r="O159" s="4"/>
+    </row>
+    <row r="160" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B160" s="16"/>
       <c r="C160" s="1" t="s">
         <v>38</v>
       </c>
@@ -6580,12 +6817,12 @@
       <c r="N160" s="6">
         <v>91</v>
       </c>
-      <c r="O160" s="10">
+      <c r="O160" s="2">
         <v>93</v>
       </c>
     </row>
-    <row r="161" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B161" s="25"/>
+    <row r="161" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B161" s="17"/>
       <c r="C161" s="3" t="s">
         <v>7</v>
       </c>
@@ -6602,10 +6839,10 @@
       <c r="L161" s="5"/>
       <c r="M161" s="4"/>
       <c r="N161" s="5"/>
-      <c r="O161" s="11"/>
-    </row>
-    <row r="162" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B162" s="24"/>
+      <c r="O161" s="4"/>
+    </row>
+    <row r="162" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B162" s="16"/>
       <c r="C162" s="1" t="s">
         <v>47</v>
       </c>
@@ -6634,10 +6871,10 @@
       <c r="N162" s="6">
         <v>1</v>
       </c>
-      <c r="O162" s="10"/>
-    </row>
-    <row r="163" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B163" s="25"/>
+      <c r="O162" s="2"/>
+    </row>
+    <row r="163" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B163" s="17"/>
       <c r="C163" s="3" t="s">
         <v>6</v>
       </c>
@@ -6666,52 +6903,55 @@
       <c r="N163" s="5">
         <v>1</v>
       </c>
-      <c r="O163" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="164" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B164" s="28"/>
-      <c r="C164" s="12" t="s">
+      <c r="O163" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B164" s="23"/>
+      <c r="C164" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D164" s="13">
-        <v>2</v>
-      </c>
-      <c r="E164" s="14">
-        <v>1</v>
-      </c>
-      <c r="F164" s="13"/>
-      <c r="G164" s="14">
-        <v>1</v>
-      </c>
-      <c r="H164" s="13">
-        <v>1</v>
-      </c>
-      <c r="I164" s="14"/>
-      <c r="J164" s="13">
-        <v>1</v>
-      </c>
-      <c r="K164" s="14">
-        <v>1</v>
-      </c>
-      <c r="L164" s="13">
-        <v>2</v>
-      </c>
-      <c r="M164" s="14">
-        <v>1</v>
-      </c>
-      <c r="N164" s="13"/>
-      <c r="O164" s="15"/>
-    </row>
-    <row r="166" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B166" s="29" t="s">
+      <c r="D164" s="25">
+        <v>2</v>
+      </c>
+      <c r="E164" s="26">
+        <v>1</v>
+      </c>
+      <c r="F164" s="25"/>
+      <c r="G164" s="26">
+        <v>1</v>
+      </c>
+      <c r="H164" s="25">
+        <v>1</v>
+      </c>
+      <c r="I164" s="26"/>
+      <c r="J164" s="25">
+        <v>1</v>
+      </c>
+      <c r="K164" s="26">
+        <v>1</v>
+      </c>
+      <c r="L164" s="25">
+        <v>2</v>
+      </c>
+      <c r="M164" s="26">
+        <v>1</v>
+      </c>
+      <c r="N164" s="25"/>
+      <c r="O164" s="26"/>
+    </row>
+    <row r="166" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B166" s="15" t="s">
         <v>56</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs: Power query ETL tips
</commit_message>
<xml_diff>
--- a/Proyectos/Proyecto8 - Funciones Adicionales de Power BI/Recursos/1+-+Ejemplos/E1.xlsx
+++ b/Proyectos/Proyecto8 - Funciones Adicionales de Power BI/Recursos/1+-+Ejemplos/E1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\Computacion\Data\Analytics\Udemy\Power BI\Curso Power BI – Análisis de Datos y Business Intelligence\Proyectos\Proyecto8 - Funciones Adicionales de Power BI\Recursos\1+-+Ejemplos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647CB4C0-9C15-460E-81C2-E3B41D5D03A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA0540C-B33C-4E97-89F5-D17E75532978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="58">
   <si>
     <t>Entertainment</t>
   </si>
@@ -191,6 +191,9 @@
   </si>
   <si>
     <t>*** Este es un resumen de la siguiente fuente: https://www.kaggle.com/tristan581/17k-apple-app-store-strategy-games</t>
+  </si>
+  <si>
+    <t>Power bi</t>
   </si>
 </sst>
 </file>
@@ -1016,25 +1019,6 @@
   </cellStyles>
   <dxfs count="17">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
@@ -1274,13 +1258,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color theme="1" tint="0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color indexed="64"/>
         </left>
@@ -1294,6 +1271,32 @@
           <color indexed="64"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1" tint="0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1309,23 +1312,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B8048242-E604-4C79-81A5-6CE7BDC5CC6E}" name="Tabla1" displayName="Tabla1" ref="B3:O164" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="15" tableBorderDxfId="16">
-  <autoFilter ref="B3:O164" xr:uid="{B8048242-E604-4C79-81A5-6CE7BDC5CC6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B8048242-E604-4C79-81A5-6CE7BDC5CC6E}" name="TablaVideoJuegos" displayName="TablaVideoJuegos" ref="B3:O197" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14">
+  <autoFilter ref="B3:O197" xr:uid="{B8048242-E604-4C79-81A5-6CE7BDC5CC6E}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{AC5C5D0F-CAE8-4FD5-824F-894A9C60453C}" name="Año" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{263B5DCD-2378-4EE1-8B13-E20479234E6B}" name="Genero" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{8D465A32-34E6-456D-93DA-5CEB86B3052D}" name="ene" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{5819C185-245E-4A38-A4D9-C4910CBA8A3B}" name="feb" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{CD859846-B5E5-4F7F-B3F1-B5F75924BD96}" name="mar" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{532140CA-633B-4570-A2B0-3B6C32434907}" name="abr" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{738A6195-FB87-482B-9667-F8D3C7AE523B}" name="may" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{0DD6B93F-117D-491A-B2CA-F8F7E9DF1601}" name="jun" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{7896AEAA-5187-42D6-9F87-F853C699F72B}" name="jul" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{AF8479E3-135F-4D22-B502-B329B86E98DD}" name="ago" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{4AE23149-1CE0-4011-A10C-EF15A68D8019}" name="sep" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{B2EA346E-0EC4-4F57-949C-B57CF4D2B578}" name="oct" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{33B998A0-7810-4531-95A3-B781D73632E9}" name="nov" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{C75CFE35-446F-40C3-A104-FF25DFABCC1F}" name="dic" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{AC5C5D0F-CAE8-4FD5-824F-894A9C60453C}" name="Año" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{263B5DCD-2378-4EE1-8B13-E20479234E6B}" name="Genero" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{8D465A32-34E6-456D-93DA-5CEB86B3052D}" name="ene" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{5819C185-245E-4A38-A4D9-C4910CBA8A3B}" name="feb" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{CD859846-B5E5-4F7F-B3F1-B5F75924BD96}" name="mar" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{532140CA-633B-4570-A2B0-3B6C32434907}" name="abr" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{738A6195-FB87-482B-9667-F8D3C7AE523B}" name="may" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{0DD6B93F-117D-491A-B2CA-F8F7E9DF1601}" name="jun" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{7896AEAA-5187-42D6-9F87-F853C699F72B}" name="jul" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{AF8479E3-135F-4D22-B502-B329B86E98DD}" name="ago" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{4AE23149-1CE0-4011-A10C-EF15A68D8019}" name="sep" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B2EA346E-0EC4-4F57-949C-B57CF4D2B578}" name="oct" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{33B998A0-7810-4531-95A3-B781D73632E9}" name="nov" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{C75CFE35-446F-40C3-A104-FF25DFABCC1F}" name="dic" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1594,7 +1597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:T166"/>
+  <dimension ref="B1:W198"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -1614,7 +1617,7 @@
     <col min="19" max="19" width="8.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="7"/>
       <c r="C1" s="7" t="s">
         <v>52</v>
@@ -1632,8 +1635,8 @@
       <c r="N1" s="7"/>
       <c r="O1" s="7"/>
     </row>
-    <row r="2" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="20" t="s">
         <v>53</v>
       </c>
@@ -1683,7 +1686,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B4" s="16" t="s">
         <v>33</v>
       </c>
@@ -1733,7 +1736,7 @@
         <v>1876</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B5" s="17"/>
       <c r="C5" s="3" t="s">
         <v>44</v>
@@ -1779,7 +1782,7 @@
         <v>2190</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B6" s="16"/>
       <c r="C6" s="1" t="s">
         <v>39</v>
@@ -1827,7 +1830,7 @@
         <v>3099</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B7" s="17"/>
       <c r="C7" s="3" t="s">
         <v>49</v>
@@ -1859,7 +1862,7 @@
         <v>2793</v>
       </c>
     </row>
-    <row r="8" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="16"/>
       <c r="C8" s="1" t="s">
         <v>10</v>
@@ -1885,7 +1888,7 @@
         <v>2484</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B9" s="17"/>
       <c r="C9" s="3" t="s">
         <v>41</v>
@@ -1927,7 +1930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B10" s="16"/>
       <c r="C10" s="1" t="s">
         <v>46</v>
@@ -1947,7 +1950,7 @@
       <c r="N10" s="6"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B11" s="17"/>
       <c r="C11" s="3" t="s">
         <v>40</v>
@@ -1989,7 +1992,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B12" s="16"/>
       <c r="C12" s="1" t="s">
         <v>5</v>
@@ -2029,7 +2032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B13" s="17"/>
       <c r="C13" s="3" t="s">
         <v>0</v>
@@ -2070,8 +2073,11 @@
       <c r="O13" s="4">
         <v>29</v>
       </c>
-    </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="R13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B14" s="16"/>
       <c r="C14" s="1" t="s">
         <v>42</v>
@@ -2113,7 +2119,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="17"/>
       <c r="C15" s="3" t="s">
         <v>16</v>
@@ -2137,7 +2143,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="16"/>
       <c r="C16" s="1" t="s">
         <v>13</v>
@@ -2160,8 +2166,14 @@
       </c>
       <c r="N16" s="6"/>
       <c r="O16" s="2"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="V16" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="W16" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B17" s="17"/>
       <c r="C17" s="3" t="s">
         <v>9</v>
@@ -2188,8 +2200,14 @@
         <v>1</v>
       </c>
       <c r="O17" s="4"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="V17" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="W17" s="9">
+        <v>1876</v>
+      </c>
+    </row>
+    <row r="18" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B18" s="16"/>
       <c r="C18" s="1" t="s">
         <v>4</v>
@@ -2208,8 +2226,14 @@
       <c r="M18" s="2"/>
       <c r="N18" s="6"/>
       <c r="O18" s="2"/>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="V18" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="W18" s="10">
+        <v>2190</v>
+      </c>
+    </row>
+    <row r="19" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B19" s="17"/>
       <c r="C19" s="3" t="s">
         <v>14</v>
@@ -2232,8 +2256,14 @@
       </c>
       <c r="N19" s="5"/>
       <c r="O19" s="4"/>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="V19" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="W19" s="9">
+        <v>3099</v>
+      </c>
+    </row>
+    <row r="20" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B20" s="16"/>
       <c r="C20" s="1" t="s">
         <v>19</v>
@@ -2254,8 +2284,14 @@
       </c>
       <c r="N20" s="6"/>
       <c r="O20" s="2"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="V20" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="W20" s="10">
+        <v>2793</v>
+      </c>
+    </row>
+    <row r="21" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="17"/>
       <c r="C21" s="3" t="s">
         <v>11</v>
@@ -2276,8 +2312,14 @@
       </c>
       <c r="N21" s="5"/>
       <c r="O21" s="4"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="V21" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="W21" s="11">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="22" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B22" s="16"/>
       <c r="C22" s="1" t="s">
         <v>8</v>
@@ -2299,7 +2341,7 @@
       <c r="N22" s="6"/>
       <c r="O22" s="2"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B23" s="17"/>
       <c r="C23" s="3" t="s">
         <v>20</v>
@@ -2341,7 +2383,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B24" s="16"/>
       <c r="C24" s="1" t="s">
         <v>50</v>
@@ -2373,7 +2415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B25" s="17"/>
       <c r="C25" s="3" t="s">
         <v>3</v>
@@ -2399,7 +2441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B26" s="16"/>
       <c r="C26" s="1" t="s">
         <v>18</v>
@@ -2441,7 +2483,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B27" s="17"/>
       <c r="C27" s="3" t="s">
         <v>45</v>
@@ -2483,7 +2525,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B28" s="16"/>
       <c r="C28" s="1" t="s">
         <v>12</v>
@@ -2511,7 +2553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B29" s="17"/>
       <c r="C29" s="3" t="s">
         <v>2</v>
@@ -2553,7 +2595,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B30" s="16"/>
       <c r="C30" s="1" t="s">
         <v>38</v>
@@ -2595,7 +2637,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B31" s="17"/>
       <c r="C31" s="3" t="s">
         <v>7</v>
@@ -2617,7 +2659,7 @@
       <c r="N31" s="5"/>
       <c r="O31" s="4"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B32" s="16"/>
       <c r="C32" s="1" t="s">
         <v>47</v>
@@ -6941,8 +6983,1070 @@
       <c r="N164" s="25"/>
       <c r="O164" s="26"/>
     </row>
+    <row r="165" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B165" s="23">
+        <v>2019</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D165" s="6">
+        <v>11</v>
+      </c>
+      <c r="E165" s="2">
+        <v>8</v>
+      </c>
+      <c r="F165" s="6">
+        <v>15</v>
+      </c>
+      <c r="G165" s="2">
+        <v>5</v>
+      </c>
+      <c r="H165" s="6">
+        <v>11</v>
+      </c>
+      <c r="I165" s="2">
+        <v>8</v>
+      </c>
+      <c r="J165" s="6">
+        <v>6</v>
+      </c>
+      <c r="K165" s="2">
+        <v>15</v>
+      </c>
+      <c r="L165" s="6">
+        <v>9</v>
+      </c>
+      <c r="M165" s="2">
+        <v>20</v>
+      </c>
+      <c r="N165" s="6">
+        <v>15</v>
+      </c>
+      <c r="O165" s="2">
+        <v>12</v>
+      </c>
+    </row>
     <row r="166" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B166" s="15" t="s">
+      <c r="B166" s="16"/>
+      <c r="C166" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D166" s="5">
+        <v>9</v>
+      </c>
+      <c r="E166" s="4">
+        <v>4</v>
+      </c>
+      <c r="F166" s="5">
+        <v>5</v>
+      </c>
+      <c r="G166" s="4">
+        <v>4</v>
+      </c>
+      <c r="H166" s="5">
+        <v>2</v>
+      </c>
+      <c r="I166" s="4">
+        <v>2</v>
+      </c>
+      <c r="J166" s="5">
+        <v>7</v>
+      </c>
+      <c r="K166" s="4">
+        <v>4</v>
+      </c>
+      <c r="L166" s="5">
+        <v>2</v>
+      </c>
+      <c r="M166" s="4">
+        <v>5</v>
+      </c>
+      <c r="N166" s="5">
+        <v>1</v>
+      </c>
+      <c r="O166" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B167" s="16"/>
+      <c r="C167" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D167" s="6">
+        <v>5</v>
+      </c>
+      <c r="E167" s="2">
+        <v>9</v>
+      </c>
+      <c r="F167" s="6">
+        <v>6</v>
+      </c>
+      <c r="G167" s="2">
+        <v>6</v>
+      </c>
+      <c r="H167" s="6">
+        <v>3</v>
+      </c>
+      <c r="I167" s="2">
+        <v>3</v>
+      </c>
+      <c r="J167" s="6">
+        <v>6</v>
+      </c>
+      <c r="K167" s="2">
+        <v>9</v>
+      </c>
+      <c r="L167" s="6">
+        <v>3</v>
+      </c>
+      <c r="M167" s="2">
+        <v>14</v>
+      </c>
+      <c r="N167" s="6">
+        <v>8</v>
+      </c>
+      <c r="O167" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="168" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B168" s="16"/>
+      <c r="C168" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D168" s="5"/>
+      <c r="E168" s="4">
+        <v>1</v>
+      </c>
+      <c r="F168" s="5"/>
+      <c r="G168" s="4"/>
+      <c r="H168" s="5">
+        <v>1</v>
+      </c>
+      <c r="I168" s="4"/>
+      <c r="J168" s="5">
+        <v>1</v>
+      </c>
+      <c r="K168" s="4">
+        <v>1</v>
+      </c>
+      <c r="L168" s="5"/>
+      <c r="M168" s="4"/>
+      <c r="N168" s="5">
+        <v>1</v>
+      </c>
+      <c r="O168" s="4"/>
+    </row>
+    <row r="169" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B169" s="16"/>
+      <c r="C169" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D169" s="6">
+        <v>1</v>
+      </c>
+      <c r="E169" s="2"/>
+      <c r="F169" s="6"/>
+      <c r="G169" s="2">
+        <v>2</v>
+      </c>
+      <c r="H169" s="6"/>
+      <c r="I169" s="2"/>
+      <c r="J169" s="6"/>
+      <c r="K169" s="2"/>
+      <c r="L169" s="6"/>
+      <c r="M169" s="2">
+        <v>1</v>
+      </c>
+      <c r="N169" s="6"/>
+      <c r="O169" s="2"/>
+    </row>
+    <row r="170" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B170" s="16"/>
+      <c r="C170" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D170" s="5">
+        <v>1</v>
+      </c>
+      <c r="E170" s="4">
+        <v>2</v>
+      </c>
+      <c r="F170" s="5">
+        <v>3</v>
+      </c>
+      <c r="G170" s="4"/>
+      <c r="H170" s="5">
+        <v>4</v>
+      </c>
+      <c r="I170" s="4"/>
+      <c r="J170" s="5">
+        <v>1</v>
+      </c>
+      <c r="K170" s="4">
+        <v>4</v>
+      </c>
+      <c r="L170" s="5">
+        <v>3</v>
+      </c>
+      <c r="M170" s="4">
+        <v>5</v>
+      </c>
+      <c r="N170" s="5">
+        <v>4</v>
+      </c>
+      <c r="O170" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="171" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B171" s="16"/>
+      <c r="C171" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D171" s="6">
+        <v>1</v>
+      </c>
+      <c r="E171" s="2">
+        <v>1</v>
+      </c>
+      <c r="F171" s="6"/>
+      <c r="G171" s="2"/>
+      <c r="H171" s="6"/>
+      <c r="I171" s="2"/>
+      <c r="J171" s="6"/>
+      <c r="K171" s="2">
+        <v>1</v>
+      </c>
+      <c r="L171" s="6">
+        <v>1</v>
+      </c>
+      <c r="M171" s="2">
+        <v>2</v>
+      </c>
+      <c r="N171" s="6"/>
+      <c r="O171" s="2"/>
+    </row>
+    <row r="172" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B172" s="16"/>
+      <c r="C172" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D172" s="5">
+        <v>12</v>
+      </c>
+      <c r="E172" s="4">
+        <v>11</v>
+      </c>
+      <c r="F172" s="5">
+        <v>7</v>
+      </c>
+      <c r="G172" s="4">
+        <v>7</v>
+      </c>
+      <c r="H172" s="5">
+        <v>4</v>
+      </c>
+      <c r="I172" s="4">
+        <v>8</v>
+      </c>
+      <c r="J172" s="5">
+        <v>13</v>
+      </c>
+      <c r="K172" s="4">
+        <v>17</v>
+      </c>
+      <c r="L172" s="5">
+        <v>8</v>
+      </c>
+      <c r="M172" s="4">
+        <v>15</v>
+      </c>
+      <c r="N172" s="5">
+        <v>15</v>
+      </c>
+      <c r="O172" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="173" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B173" s="16"/>
+      <c r="C173" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D173" s="6">
+        <v>6</v>
+      </c>
+      <c r="E173" s="2">
+        <v>10</v>
+      </c>
+      <c r="F173" s="6">
+        <v>14</v>
+      </c>
+      <c r="G173" s="2">
+        <v>6</v>
+      </c>
+      <c r="H173" s="6">
+        <v>4</v>
+      </c>
+      <c r="I173" s="2">
+        <v>3</v>
+      </c>
+      <c r="J173" s="6">
+        <v>11</v>
+      </c>
+      <c r="K173" s="2">
+        <v>7</v>
+      </c>
+      <c r="L173" s="6">
+        <v>8</v>
+      </c>
+      <c r="M173" s="2">
+        <v>11</v>
+      </c>
+      <c r="N173" s="6">
+        <v>6</v>
+      </c>
+      <c r="O173" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="174" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B174" s="16"/>
+      <c r="C174" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D174" s="5">
+        <v>18</v>
+      </c>
+      <c r="E174" s="4">
+        <v>18</v>
+      </c>
+      <c r="F174" s="5">
+        <v>26</v>
+      </c>
+      <c r="G174" s="4">
+        <v>20</v>
+      </c>
+      <c r="H174" s="5">
+        <v>17</v>
+      </c>
+      <c r="I174" s="4">
+        <v>22</v>
+      </c>
+      <c r="J174" s="5">
+        <v>39</v>
+      </c>
+      <c r="K174" s="4">
+        <v>49</v>
+      </c>
+      <c r="L174" s="5">
+        <v>31</v>
+      </c>
+      <c r="M174" s="4">
+        <v>25</v>
+      </c>
+      <c r="N174" s="5">
+        <v>29</v>
+      </c>
+      <c r="O174" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="175" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B175" s="16"/>
+      <c r="C175" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D175" s="6"/>
+      <c r="E175" s="2">
+        <v>2</v>
+      </c>
+      <c r="F175" s="6">
+        <v>2</v>
+      </c>
+      <c r="G175" s="2">
+        <v>3</v>
+      </c>
+      <c r="H175" s="6"/>
+      <c r="I175" s="2">
+        <v>1</v>
+      </c>
+      <c r="J175" s="6">
+        <v>4</v>
+      </c>
+      <c r="K175" s="2">
+        <v>3</v>
+      </c>
+      <c r="L175" s="6">
+        <v>2</v>
+      </c>
+      <c r="M175" s="2">
+        <v>5</v>
+      </c>
+      <c r="N175" s="6"/>
+      <c r="O175" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B176" s="16"/>
+      <c r="C176" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D176" s="5"/>
+      <c r="E176" s="4"/>
+      <c r="F176" s="5">
+        <v>1</v>
+      </c>
+      <c r="G176" s="4">
+        <v>1</v>
+      </c>
+      <c r="H176" s="5">
+        <v>1</v>
+      </c>
+      <c r="I176" s="4"/>
+      <c r="J176" s="5"/>
+      <c r="K176" s="4"/>
+      <c r="L176" s="5"/>
+      <c r="M176" s="4"/>
+      <c r="N176" s="5"/>
+      <c r="O176" s="4"/>
+    </row>
+    <row r="177" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B177" s="16"/>
+      <c r="C177" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D177" s="6"/>
+      <c r="E177" s="2"/>
+      <c r="F177" s="6">
+        <v>1</v>
+      </c>
+      <c r="G177" s="2"/>
+      <c r="H177" s="6"/>
+      <c r="I177" s="2"/>
+      <c r="J177" s="6">
+        <v>1</v>
+      </c>
+      <c r="K177" s="2">
+        <v>2</v>
+      </c>
+      <c r="L177" s="6"/>
+      <c r="M177" s="2"/>
+      <c r="N177" s="6"/>
+      <c r="O177" s="2"/>
+    </row>
+    <row r="178" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B178" s="16"/>
+      <c r="C178" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D178" s="5"/>
+      <c r="E178" s="4"/>
+      <c r="F178" s="5"/>
+      <c r="G178" s="4">
+        <v>1</v>
+      </c>
+      <c r="H178" s="5"/>
+      <c r="I178" s="4"/>
+      <c r="J178" s="5"/>
+      <c r="K178" s="4"/>
+      <c r="L178" s="5"/>
+      <c r="M178" s="4">
+        <v>2</v>
+      </c>
+      <c r="N178" s="5"/>
+      <c r="O178" s="4"/>
+    </row>
+    <row r="179" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B179" s="16"/>
+      <c r="C179" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D179" s="6">
+        <v>1</v>
+      </c>
+      <c r="E179" s="2">
+        <v>1</v>
+      </c>
+      <c r="F179" s="6">
+        <v>1</v>
+      </c>
+      <c r="G179" s="2">
+        <v>2</v>
+      </c>
+      <c r="H179" s="6">
+        <v>1</v>
+      </c>
+      <c r="I179" s="2"/>
+      <c r="J179" s="6">
+        <v>2</v>
+      </c>
+      <c r="K179" s="2">
+        <v>2</v>
+      </c>
+      <c r="L179" s="6">
+        <v>3</v>
+      </c>
+      <c r="M179" s="2">
+        <v>3</v>
+      </c>
+      <c r="N179" s="6">
+        <v>2</v>
+      </c>
+      <c r="O179" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="180" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B180" s="16"/>
+      <c r="C180" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D180" s="5"/>
+      <c r="E180" s="4"/>
+      <c r="F180" s="5"/>
+      <c r="G180" s="4">
+        <v>1</v>
+      </c>
+      <c r="H180" s="5"/>
+      <c r="I180" s="4"/>
+      <c r="J180" s="5"/>
+      <c r="K180" s="4">
+        <v>1</v>
+      </c>
+      <c r="L180" s="5">
+        <v>2</v>
+      </c>
+      <c r="M180" s="4"/>
+      <c r="N180" s="5">
+        <v>2</v>
+      </c>
+      <c r="O180" s="4"/>
+    </row>
+    <row r="181" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B181" s="16"/>
+      <c r="C181" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D181" s="6"/>
+      <c r="E181" s="2"/>
+      <c r="F181" s="6"/>
+      <c r="G181" s="2"/>
+      <c r="H181" s="6"/>
+      <c r="I181" s="2"/>
+      <c r="J181" s="6">
+        <v>2</v>
+      </c>
+      <c r="K181" s="2"/>
+      <c r="L181" s="6"/>
+      <c r="M181" s="2"/>
+      <c r="N181" s="6">
+        <v>1</v>
+      </c>
+      <c r="O181" s="2"/>
+    </row>
+    <row r="182" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B182" s="16"/>
+      <c r="C182" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D182" s="5"/>
+      <c r="E182" s="4"/>
+      <c r="F182" s="5"/>
+      <c r="G182" s="4"/>
+      <c r="H182" s="5"/>
+      <c r="I182" s="4"/>
+      <c r="J182" s="5">
+        <v>1</v>
+      </c>
+      <c r="K182" s="4"/>
+      <c r="L182" s="5"/>
+      <c r="M182" s="4"/>
+      <c r="N182" s="5"/>
+      <c r="O182" s="4"/>
+    </row>
+    <row r="183" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B183" s="16"/>
+      <c r="C183" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D183" s="6"/>
+      <c r="E183" s="2"/>
+      <c r="F183" s="6"/>
+      <c r="G183" s="2"/>
+      <c r="H183" s="6"/>
+      <c r="I183" s="2"/>
+      <c r="J183" s="6"/>
+      <c r="K183" s="2"/>
+      <c r="L183" s="6"/>
+      <c r="M183" s="2"/>
+      <c r="N183" s="6">
+        <v>1</v>
+      </c>
+      <c r="O183" s="2"/>
+    </row>
+    <row r="184" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B184" s="16"/>
+      <c r="C184" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D184" s="5"/>
+      <c r="E184" s="4">
+        <v>1</v>
+      </c>
+      <c r="F184" s="5"/>
+      <c r="G184" s="4">
+        <v>1</v>
+      </c>
+      <c r="H184" s="5"/>
+      <c r="I184" s="4"/>
+      <c r="J184" s="5">
+        <v>1</v>
+      </c>
+      <c r="K184" s="4"/>
+      <c r="L184" s="5"/>
+      <c r="M184" s="4"/>
+      <c r="N184" s="5">
+        <v>1</v>
+      </c>
+      <c r="O184" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="185" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B185" s="16"/>
+      <c r="C185" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D185" s="6">
+        <v>20</v>
+      </c>
+      <c r="E185" s="2">
+        <v>20</v>
+      </c>
+      <c r="F185" s="6">
+        <v>18</v>
+      </c>
+      <c r="G185" s="2">
+        <v>12</v>
+      </c>
+      <c r="H185" s="6">
+        <v>8</v>
+      </c>
+      <c r="I185" s="2">
+        <v>11</v>
+      </c>
+      <c r="J185" s="6">
+        <v>16</v>
+      </c>
+      <c r="K185" s="2">
+        <v>28</v>
+      </c>
+      <c r="L185" s="6">
+        <v>18</v>
+      </c>
+      <c r="M185" s="2">
+        <v>19</v>
+      </c>
+      <c r="N185" s="6">
+        <v>18</v>
+      </c>
+      <c r="O185" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="186" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B186" s="16"/>
+      <c r="C186" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D186" s="5"/>
+      <c r="E186" s="4">
+        <v>1</v>
+      </c>
+      <c r="F186" s="5">
+        <v>1</v>
+      </c>
+      <c r="G186" s="4"/>
+      <c r="H186" s="5"/>
+      <c r="I186" s="4"/>
+      <c r="J186" s="5"/>
+      <c r="K186" s="4"/>
+      <c r="L186" s="5"/>
+      <c r="M186" s="4"/>
+      <c r="N186" s="5"/>
+      <c r="O186" s="4"/>
+    </row>
+    <row r="187" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B187" s="16"/>
+      <c r="C187" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D187" s="6"/>
+      <c r="E187" s="2"/>
+      <c r="F187" s="6">
+        <v>1</v>
+      </c>
+      <c r="G187" s="2"/>
+      <c r="H187" s="6">
+        <v>1</v>
+      </c>
+      <c r="I187" s="2"/>
+      <c r="J187" s="6"/>
+      <c r="K187" s="2">
+        <v>1</v>
+      </c>
+      <c r="L187" s="6"/>
+      <c r="M187" s="2"/>
+      <c r="N187" s="6"/>
+      <c r="O187" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B188" s="16"/>
+      <c r="C188" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D188" s="5">
+        <v>5</v>
+      </c>
+      <c r="E188" s="4">
+        <v>2</v>
+      </c>
+      <c r="F188" s="5">
+        <v>8</v>
+      </c>
+      <c r="G188" s="4">
+        <v>6</v>
+      </c>
+      <c r="H188" s="5">
+        <v>6</v>
+      </c>
+      <c r="I188" s="4">
+        <v>5</v>
+      </c>
+      <c r="J188" s="5">
+        <v>7</v>
+      </c>
+      <c r="K188" s="4">
+        <v>8</v>
+      </c>
+      <c r="L188" s="5">
+        <v>9</v>
+      </c>
+      <c r="M188" s="4">
+        <v>4</v>
+      </c>
+      <c r="N188" s="5">
+        <v>2</v>
+      </c>
+      <c r="O188" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="189" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B189" s="16"/>
+      <c r="C189" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D189" s="6">
+        <v>15</v>
+      </c>
+      <c r="E189" s="2">
+        <v>15</v>
+      </c>
+      <c r="F189" s="6">
+        <v>9</v>
+      </c>
+      <c r="G189" s="2">
+        <v>12</v>
+      </c>
+      <c r="H189" s="6">
+        <v>13</v>
+      </c>
+      <c r="I189" s="2">
+        <v>7</v>
+      </c>
+      <c r="J189" s="6">
+        <v>17</v>
+      </c>
+      <c r="K189" s="2">
+        <v>18</v>
+      </c>
+      <c r="L189" s="6">
+        <v>8</v>
+      </c>
+      <c r="M189" s="2">
+        <v>7</v>
+      </c>
+      <c r="N189" s="6">
+        <v>13</v>
+      </c>
+      <c r="O189" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="190" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B190" s="16"/>
+      <c r="C190" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D190" s="5">
+        <v>1</v>
+      </c>
+      <c r="E190" s="4"/>
+      <c r="F190" s="5">
+        <v>2</v>
+      </c>
+      <c r="G190" s="4">
+        <v>1</v>
+      </c>
+      <c r="H190" s="5"/>
+      <c r="I190" s="4"/>
+      <c r="J190" s="5">
+        <v>2</v>
+      </c>
+      <c r="K190" s="4">
+        <v>2</v>
+      </c>
+      <c r="L190" s="5">
+        <v>1</v>
+      </c>
+      <c r="M190" s="4"/>
+      <c r="N190" s="5"/>
+      <c r="O190" s="4"/>
+    </row>
+    <row r="191" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B191" s="16"/>
+      <c r="C191" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D191" s="6">
+        <v>1</v>
+      </c>
+      <c r="E191" s="2">
+        <v>4</v>
+      </c>
+      <c r="F191" s="6">
+        <v>3</v>
+      </c>
+      <c r="G191" s="2">
+        <v>5</v>
+      </c>
+      <c r="H191" s="6">
+        <v>1</v>
+      </c>
+      <c r="I191" s="2">
+        <v>10</v>
+      </c>
+      <c r="J191" s="6">
+        <v>6</v>
+      </c>
+      <c r="K191" s="2">
+        <v>6</v>
+      </c>
+      <c r="L191" s="6">
+        <v>4</v>
+      </c>
+      <c r="M191" s="2">
+        <v>5</v>
+      </c>
+      <c r="N191" s="6">
+        <v>2</v>
+      </c>
+      <c r="O191" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="192" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B192" s="16"/>
+      <c r="C192" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D192" s="5"/>
+      <c r="E192" s="4"/>
+      <c r="F192" s="5"/>
+      <c r="G192" s="4">
+        <v>1</v>
+      </c>
+      <c r="H192" s="5"/>
+      <c r="I192" s="4"/>
+      <c r="J192" s="5"/>
+      <c r="K192" s="4"/>
+      <c r="L192" s="5"/>
+      <c r="M192" s="4"/>
+      <c r="N192" s="5"/>
+      <c r="O192" s="4"/>
+    </row>
+    <row r="193" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B193" s="16"/>
+      <c r="C193" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D193" s="6">
+        <v>78</v>
+      </c>
+      <c r="E193" s="2">
+        <v>82</v>
+      </c>
+      <c r="F193" s="6">
+        <v>87</v>
+      </c>
+      <c r="G193" s="2">
+        <v>84</v>
+      </c>
+      <c r="H193" s="6">
+        <v>62</v>
+      </c>
+      <c r="I193" s="2">
+        <v>51</v>
+      </c>
+      <c r="J193" s="6">
+        <v>100</v>
+      </c>
+      <c r="K193" s="2">
+        <v>143</v>
+      </c>
+      <c r="L193" s="6">
+        <v>88</v>
+      </c>
+      <c r="M193" s="2">
+        <v>83</v>
+      </c>
+      <c r="N193" s="6">
+        <v>91</v>
+      </c>
+      <c r="O193" s="2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="194" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B194" s="16"/>
+      <c r="C194" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D194" s="5"/>
+      <c r="E194" s="4">
+        <v>1</v>
+      </c>
+      <c r="F194" s="5"/>
+      <c r="G194" s="4"/>
+      <c r="H194" s="5"/>
+      <c r="I194" s="4"/>
+      <c r="J194" s="5"/>
+      <c r="K194" s="4"/>
+      <c r="L194" s="5"/>
+      <c r="M194" s="4"/>
+      <c r="N194" s="5"/>
+      <c r="O194" s="4"/>
+    </row>
+    <row r="195" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B195" s="16"/>
+      <c r="C195" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D195" s="6"/>
+      <c r="E195" s="2">
+        <v>1</v>
+      </c>
+      <c r="F195" s="6">
+        <v>2</v>
+      </c>
+      <c r="G195" s="2">
+        <v>1</v>
+      </c>
+      <c r="H195" s="6"/>
+      <c r="I195" s="2"/>
+      <c r="J195" s="6"/>
+      <c r="K195" s="2">
+        <v>1</v>
+      </c>
+      <c r="L195" s="6">
+        <v>1</v>
+      </c>
+      <c r="M195" s="2">
+        <v>2</v>
+      </c>
+      <c r="N195" s="6">
+        <v>1</v>
+      </c>
+      <c r="O195" s="2"/>
+    </row>
+    <row r="196" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B196" s="16"/>
+      <c r="C196" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D196" s="5">
+        <v>1</v>
+      </c>
+      <c r="E196" s="4">
+        <v>1</v>
+      </c>
+      <c r="F196" s="5"/>
+      <c r="G196" s="4"/>
+      <c r="H196" s="5"/>
+      <c r="I196" s="4"/>
+      <c r="J196" s="5">
+        <v>1</v>
+      </c>
+      <c r="K196" s="4">
+        <v>2</v>
+      </c>
+      <c r="L196" s="5">
+        <v>3</v>
+      </c>
+      <c r="M196" s="4">
+        <v>2</v>
+      </c>
+      <c r="N196" s="5">
+        <v>1</v>
+      </c>
+      <c r="O196" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="197" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B197" s="16"/>
+      <c r="C197" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="D197" s="25">
+        <v>2</v>
+      </c>
+      <c r="E197" s="26">
+        <v>1</v>
+      </c>
+      <c r="F197" s="25"/>
+      <c r="G197" s="26">
+        <v>1</v>
+      </c>
+      <c r="H197" s="25">
+        <v>1</v>
+      </c>
+      <c r="I197" s="26"/>
+      <c r="J197" s="25">
+        <v>1</v>
+      </c>
+      <c r="K197" s="26">
+        <v>1</v>
+      </c>
+      <c r="L197" s="25">
+        <v>2</v>
+      </c>
+      <c r="M197" s="26">
+        <v>1</v>
+      </c>
+      <c r="N197" s="25"/>
+      <c r="O197" s="26"/>
+    </row>
+    <row r="198" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B198" s="15" t="s">
         <v>56</v>
       </c>
     </row>

</xml_diff>